<commit_message>
feat: Week 21 · Supply unificado + Excels consolidados · 19-25 mayo 2026
Pipeline completo W21: calc → render → assemble_unified → excel (4 hojas) → mail → hub → docs → commit
</commit_message>
<xml_diff>
--- a/checkrates/week-21/Analisis_CheckRates_W21.xlsx
+++ b/checkrates/week-21/Analisis_CheckRates_W21.xlsx
@@ -555,14 +555,14 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1342 hoteles P80 · 19-25 mayo 2025</t>
+          <t>1342 hoteles P80 · 19-25 mayo 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>W21 · 19-25 mayo 2025 · Generado 26/05/2026 17:56</t>
+          <t>W21 · 19-25 mayo 2026 · Generado 26/05/2026 20:15</t>
         </is>
       </c>
     </row>
@@ -24018,14 +24018,14 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>266 hoteles P80 · 19-25 mayo 2025</t>
+          <t>266 hoteles P80 · 19-25 mayo 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>W21 · 19-25 mayo 2025 · Generado 26/05/2026 17:56</t>
+          <t>W21 · 19-25 mayo 2026 · Generado 26/05/2026 20:15</t>
         </is>
       </c>
     </row>
@@ -38117,14 +38117,14 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1051 hoteles P80 · 19-25 mayo 2025</t>
+          <t>1051 hoteles P80 · 19-25 mayo 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>W21 · 19-25 mayo 2025 · Generado 26/05/2026 17:56</t>
+          <t>W21 · 19-25 mayo 2026 · Generado 26/05/2026 20:15</t>
         </is>
       </c>
     </row>
@@ -59955,14 +59955,14 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>372 hoteles P80 · 19-25 mayo 2025</t>
+          <t>372 hoteles P80 · 19-25 mayo 2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>W21 · 19-25 mayo 2025 · Generado 26/05/2026 17:56</t>
+          <t>W21 · 19-25 mayo 2026 · Generado 26/05/2026 20:15</t>
         </is>
       </c>
     </row>

</xml_diff>